<commit_message>
feat(search-pages): each download page shows a preview of its real file
Every download page now shows its filled-in example (the Excel example
sheet or the PDF example page) at four srcset widths, with alt text
saying what it shows; the previews ship only with live pages, and admin
shows a placeholder. Made by scripts/make-download-previews.mjs (macOS:
PDFKit, Quick Look, Playwright, sharp). The Excel sheets now show every
label in column A and use Arial, and the appointment book PDF gains a
sample week. The six pages drop their last toConfirm item
(plan 2026-10-31-002, U13; #1206).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/packages/search-pages/content/downloads/files/appointment-book/appointment-book.xlsx
+++ b/packages/search-pages/content/downloads/files/appointment-book/appointment-book.xlsx
@@ -188,25 +188,25 @@
   <fonts count="4">
     <font>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF6B7280"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>

</xml_diff>